<commit_message>
adjusted start and end dates to get more accurate return numbers
</commit_message>
<xml_diff>
--- a/results-excel/backtest_results.xlsx
+++ b/results-excel/backtest_results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O27"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,65 +430,45 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>price_return</t>
+          <t>benchmark_return</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>dividend_return</t>
+          <t>active_return</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>benchmark_return</t>
+          <t>active_share</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>benchmark_price_return</t>
+          <t>max_sector_deviation</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>benchmark_dividend_return</t>
+          <t>max_ig_deviation</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>active_return</t>
+          <t>passed_sector_constraint</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>active_share</t>
+          <t>passed_ig_constraint</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>max_sector_deviation</t>
+          <t>coverage_pct</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
-        <is>
-          <t>max_ig_deviation</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>passed_sector_constraint</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>passed_ig_constraint</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>coverage_pct</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
         <is>
           <t>n_stocks</t>
         </is>
@@ -499,41 +479,33 @@
         <v>2000</v>
       </c>
       <c r="B2" t="n">
-        <v>-10.52549099620005</v>
+        <v>-12.68959958663498</v>
       </c>
       <c r="C2" t="n">
-        <v>-13.50619148981854</v>
+        <v>-9.1</v>
       </c>
       <c r="D2" t="n">
-        <v>2.979541516837573</v>
+        <v>-3.589599586634984</v>
       </c>
       <c r="E2" t="n">
-        <v>-9.1</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
-        <v>-1.425490996200052</v>
-      </c>
-      <c r="I2" t="n">
         <v>35.88174522990984</v>
       </c>
+      <c r="F2" t="n">
+        <v>2.000000000000011</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
       <c r="J2" t="n">
-        <v>2.000000000000011</v>
+        <v>100</v>
       </c>
       <c r="K2" t="n">
-        <v>2.000000000000004</v>
-      </c>
-      <c r="L2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M2" t="b">
-        <v>1</v>
-      </c>
-      <c r="N2" t="n">
-        <v>100</v>
-      </c>
-      <c r="O2" t="n">
         <v>60</v>
       </c>
     </row>
@@ -542,41 +514,33 @@
         <v>2001</v>
       </c>
       <c r="B3" t="n">
-        <v>-11.8536199604649</v>
+        <v>-13.78670946962385</v>
       </c>
       <c r="C3" t="n">
-        <v>-13.58271174917598</v>
+        <v>-11.89</v>
       </c>
       <c r="D3" t="n">
-        <v>1.726922249882319</v>
+        <v>-1.896709469623854</v>
       </c>
       <c r="E3" t="n">
-        <v>-11.89</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
-        <v>0.03638003953510172</v>
-      </c>
-      <c r="I3" t="n">
         <v>38.75841929218824</v>
       </c>
+      <c r="F3" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
       <c r="J3" t="n">
-        <v>2.000000000000002</v>
+        <v>100</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
-      </c>
-      <c r="L3" t="b">
-        <v>1</v>
-      </c>
-      <c r="M3" t="b">
-        <v>1</v>
-      </c>
-      <c r="N3" t="n">
-        <v>100</v>
-      </c>
-      <c r="O3" t="n">
         <v>60</v>
       </c>
     </row>
@@ -585,41 +549,33 @@
         <v>2002</v>
       </c>
       <c r="B4" t="n">
-        <v>-22.99911160770736</v>
+        <v>-22.8047545975154</v>
       </c>
       <c r="C4" t="n">
-        <v>-25.30241945726711</v>
+        <v>-22.1</v>
       </c>
       <c r="D4" t="n">
-        <v>2.301091523696105</v>
+        <v>-0.7047545975154001</v>
       </c>
       <c r="E4" t="n">
-        <v>-22.1</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="n">
-        <v>-0.8991116077073542</v>
-      </c>
-      <c r="I4" t="n">
         <v>40.50861655160997</v>
       </c>
+      <c r="F4" t="n">
+        <v>2.000000000000005</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2.000000000000007</v>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
       <c r="J4" t="n">
-        <v>2.000000000000005</v>
+        <v>100</v>
       </c>
       <c r="K4" t="n">
-        <v>2.000000000000007</v>
-      </c>
-      <c r="L4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M4" t="b">
-        <v>1</v>
-      </c>
-      <c r="N4" t="n">
-        <v>100</v>
-      </c>
-      <c r="O4" t="n">
         <v>60</v>
       </c>
     </row>
@@ -628,41 +584,33 @@
         <v>2003</v>
       </c>
       <c r="B5" t="n">
-        <v>23.04444600102246</v>
+        <v>25.97420939705834</v>
       </c>
       <c r="C5" t="n">
-        <v>19.71209876326909</v>
+        <v>28.68</v>
       </c>
       <c r="D5" t="n">
-        <v>3.332511002207112</v>
+        <v>-2.705790602941658</v>
       </c>
       <c r="E5" t="n">
-        <v>28.68</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
-        <v>-5.635553998977539</v>
-      </c>
-      <c r="I5" t="n">
         <v>41.02983047854167</v>
       </c>
+      <c r="F5" t="n">
+        <v>2.000000000000001</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
       <c r="J5" t="n">
-        <v>2.000000000000001</v>
+        <v>100</v>
       </c>
       <c r="K5" t="n">
-        <v>2.000000000000004</v>
-      </c>
-      <c r="L5" t="b">
-        <v>1</v>
-      </c>
-      <c r="M5" t="b">
-        <v>1</v>
-      </c>
-      <c r="N5" t="n">
-        <v>100</v>
-      </c>
-      <c r="O5" t="n">
         <v>60</v>
       </c>
     </row>
@@ -671,41 +619,33 @@
         <v>2004</v>
       </c>
       <c r="B6" t="n">
-        <v>9.977587210205572</v>
+        <v>9.388976511728519</v>
       </c>
       <c r="C6" t="n">
-        <v>6.844700039677869</v>
+        <v>10.88</v>
       </c>
       <c r="D6" t="n">
-        <v>3.130713108929453</v>
+        <v>-1.491023488271482</v>
       </c>
       <c r="E6" t="n">
-        <v>10.88</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
-        <v>-0.902412789794429</v>
-      </c>
-      <c r="I6" t="n">
         <v>43.42485340092188</v>
       </c>
+      <c r="F6" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
       <c r="J6" t="n">
-        <v>2.000000000000002</v>
+        <v>100</v>
       </c>
       <c r="K6" t="n">
-        <v>2.000000000000002</v>
-      </c>
-      <c r="L6" t="b">
-        <v>1</v>
-      </c>
-      <c r="M6" t="b">
-        <v>1</v>
-      </c>
-      <c r="N6" t="n">
-        <v>100</v>
-      </c>
-      <c r="O6" t="n">
         <v>60</v>
       </c>
     </row>
@@ -714,41 +654,33 @@
         <v>2005</v>
       </c>
       <c r="B7" t="n">
-        <v>1.933465789967272</v>
+        <v>1.382717571470944</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.8709016808749677</v>
+        <v>4.91</v>
       </c>
       <c r="D7" t="n">
-        <v>2.803904534428515</v>
+        <v>-3.527282428529056</v>
       </c>
       <c r="E7" t="n">
-        <v>4.91</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="n">
-        <v>-2.976534210032729</v>
-      </c>
-      <c r="I7" t="n">
         <v>45.53284177840612</v>
       </c>
+      <c r="F7" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
       <c r="J7" t="n">
-        <v>2.000000000000004</v>
+        <v>100</v>
       </c>
       <c r="K7" t="n">
-        <v>2.000000000000004</v>
-      </c>
-      <c r="L7" t="b">
-        <v>1</v>
-      </c>
-      <c r="M7" t="b">
-        <v>1</v>
-      </c>
-      <c r="N7" t="n">
-        <v>100</v>
-      </c>
-      <c r="O7" t="n">
         <v>60</v>
       </c>
     </row>
@@ -757,41 +689,33 @@
         <v>2006</v>
       </c>
       <c r="B8" t="n">
-        <v>13.70332558080793</v>
+        <v>16.09894671626479</v>
       </c>
       <c r="C8" t="n">
-        <v>11.14622429069041</v>
+        <v>15.79</v>
       </c>
       <c r="D8" t="n">
-        <v>2.556999929197793</v>
+        <v>0.3089467162647885</v>
       </c>
       <c r="E8" t="n">
-        <v>15.79</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="n">
-        <v>-2.086674419192072</v>
-      </c>
-      <c r="I8" t="n">
         <v>47.18838431687644</v>
       </c>
+      <c r="F8" t="n">
+        <v>2.000000000000005</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
       <c r="J8" t="n">
-        <v>2.000000000000005</v>
+        <v>100</v>
       </c>
       <c r="K8" t="n">
-        <v>2.000000000000004</v>
-      </c>
-      <c r="L8" t="b">
-        <v>1</v>
-      </c>
-      <c r="M8" t="b">
-        <v>1</v>
-      </c>
-      <c r="N8" t="n">
-        <v>100</v>
-      </c>
-      <c r="O8" t="n">
         <v>60</v>
       </c>
     </row>
@@ -800,41 +724,33 @@
         <v>2007</v>
       </c>
       <c r="B9" t="n">
-        <v>9.430931663130986</v>
+        <v>6.005867904111259</v>
       </c>
       <c r="C9" t="n">
-        <v>3.219819903382591</v>
+        <v>5.49</v>
       </c>
       <c r="D9" t="n">
-        <v>6.231250619937311</v>
+        <v>0.5158679041112588</v>
       </c>
       <c r="E9" t="n">
-        <v>5.49</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="n">
-        <v>3.940931663130986</v>
-      </c>
-      <c r="I9" t="n">
         <v>45.99605802065285</v>
       </c>
+      <c r="F9" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2.000000000000001</v>
+      </c>
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" t="b">
+        <v>1</v>
+      </c>
       <c r="J9" t="n">
-        <v>2.000000000000004</v>
+        <v>100</v>
       </c>
       <c r="K9" t="n">
-        <v>2.000000000000001</v>
-      </c>
-      <c r="L9" t="b">
-        <v>1</v>
-      </c>
-      <c r="M9" t="b">
-        <v>1</v>
-      </c>
-      <c r="N9" t="n">
-        <v>100</v>
-      </c>
-      <c r="O9" t="n">
         <v>60</v>
       </c>
     </row>
@@ -843,41 +759,33 @@
         <v>2008</v>
       </c>
       <c r="B10" t="n">
-        <v>-29.64754988133485</v>
+        <v>-33.7345293201338</v>
       </c>
       <c r="C10" t="n">
-        <v>-34.74418854468603</v>
+        <v>-37</v>
       </c>
       <c r="D10" t="n">
-        <v>5.152409164630893</v>
+        <v>3.265470679866205</v>
       </c>
       <c r="E10" t="n">
-        <v>-37</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
-        <v>7.352450118665153</v>
-      </c>
-      <c r="I10" t="n">
         <v>46.45562053681084</v>
       </c>
+      <c r="F10" t="n">
+        <v>2.000000000000001</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2.000000000000001</v>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
       <c r="J10" t="n">
-        <v>2.000000000000001</v>
+        <v>100</v>
       </c>
       <c r="K10" t="n">
-        <v>2.000000000000001</v>
-      </c>
-      <c r="L10" t="b">
-        <v>1</v>
-      </c>
-      <c r="M10" t="b">
-        <v>1</v>
-      </c>
-      <c r="N10" t="n">
-        <v>100</v>
-      </c>
-      <c r="O10" t="n">
         <v>60</v>
       </c>
     </row>
@@ -886,41 +794,33 @@
         <v>2009</v>
       </c>
       <c r="B11" t="n">
-        <v>16.97700001204536</v>
+        <v>20.72737264474318</v>
       </c>
       <c r="C11" t="n">
-        <v>13.96801122425574</v>
+        <v>26.46</v>
       </c>
       <c r="D11" t="n">
-        <v>3.009162849010612</v>
+        <v>-5.732627355256817</v>
       </c>
       <c r="E11" t="n">
-        <v>26.46</v>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="n">
-        <v>-9.482999987954646</v>
-      </c>
-      <c r="I11" t="n">
         <v>42.48514837560866</v>
       </c>
+      <c r="F11" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2.000000000000001</v>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
       <c r="J11" t="n">
-        <v>2.000000000000002</v>
+        <v>100</v>
       </c>
       <c r="K11" t="n">
-        <v>2.000000000000001</v>
-      </c>
-      <c r="L11" t="b">
-        <v>1</v>
-      </c>
-      <c r="M11" t="b">
-        <v>1</v>
-      </c>
-      <c r="N11" t="n">
-        <v>100</v>
-      </c>
-      <c r="O11" t="n">
         <v>60</v>
       </c>
     </row>
@@ -929,41 +829,33 @@
         <v>2010</v>
       </c>
       <c r="B12" t="n">
-        <v>9.19860258597023</v>
+        <v>10.858190355809</v>
       </c>
       <c r="C12" t="n">
-        <v>6.760062501035564</v>
+        <v>15.06</v>
       </c>
       <c r="D12" t="n">
-        <v>2.430992992332452</v>
+        <v>-4.201809644191004</v>
       </c>
       <c r="E12" t="n">
-        <v>15.06</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="n">
-        <v>-5.861397414029771</v>
-      </c>
-      <c r="I12" t="n">
         <v>45.17063017820425</v>
       </c>
+      <c r="F12" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
       <c r="J12" t="n">
-        <v>2.000000000000004</v>
+        <v>100</v>
       </c>
       <c r="K12" t="n">
-        <v>2.000000000000004</v>
-      </c>
-      <c r="L12" t="b">
-        <v>1</v>
-      </c>
-      <c r="M12" t="b">
-        <v>1</v>
-      </c>
-      <c r="N12" t="n">
-        <v>100</v>
-      </c>
-      <c r="O12" t="n">
         <v>60</v>
       </c>
     </row>
@@ -972,41 +864,33 @@
         <v>2011</v>
       </c>
       <c r="B13" t="n">
-        <v>2.486255929487801</v>
+        <v>3.467109693648268</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.1341393335045956</v>
+        <v>2.11</v>
       </c>
       <c r="D13" t="n">
-        <v>2.620395262992397</v>
+        <v>1.357109693648268</v>
       </c>
       <c r="E13" t="n">
-        <v>2.11</v>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="n">
-        <v>0.3762559294878014</v>
-      </c>
-      <c r="I13" t="n">
         <v>46.44260294899527</v>
       </c>
+      <c r="F13" t="n">
+        <v>2.000000000000007</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
       <c r="J13" t="n">
-        <v>2.000000000000007</v>
+        <v>100</v>
       </c>
       <c r="K13" t="n">
-        <v>2.000000000000004</v>
-      </c>
-      <c r="L13" t="b">
-        <v>1</v>
-      </c>
-      <c r="M13" t="b">
-        <v>1</v>
-      </c>
-      <c r="N13" t="n">
-        <v>100</v>
-      </c>
-      <c r="O13" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1015,41 +899,33 @@
         <v>2012</v>
       </c>
       <c r="B14" t="n">
-        <v>16.45095793784687</v>
+        <v>17.91262893932726</v>
       </c>
       <c r="C14" t="n">
-        <v>11.12673096920813</v>
+        <v>16</v>
       </c>
       <c r="D14" t="n">
-        <v>5.324226968638733</v>
+        <v>1.912628939327263</v>
       </c>
       <c r="E14" t="n">
-        <v>16</v>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="n">
-        <v>0.4509579378468658</v>
-      </c>
-      <c r="I14" t="n">
         <v>46.04995550710298</v>
       </c>
+      <c r="F14" t="n">
+        <v>1.95784686755224</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" t="b">
+        <v>1</v>
+      </c>
       <c r="J14" t="n">
-        <v>1.95784686755224</v>
+        <v>100</v>
       </c>
       <c r="K14" t="n">
-        <v>2</v>
-      </c>
-      <c r="L14" t="b">
-        <v>1</v>
-      </c>
-      <c r="M14" t="b">
-        <v>1</v>
-      </c>
-      <c r="N14" t="n">
-        <v>100</v>
-      </c>
-      <c r="O14" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1058,41 +934,33 @@
         <v>2013</v>
       </c>
       <c r="B15" t="n">
-        <v>28.79620612952294</v>
+        <v>29.1275238721401</v>
       </c>
       <c r="C15" t="n">
-        <v>23.07599060359207</v>
+        <v>32.39</v>
       </c>
       <c r="D15" t="n">
-        <v>5.720215525930871</v>
+        <v>-3.262476127859905</v>
       </c>
       <c r="E15" t="n">
-        <v>32.39</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="n">
-        <v>-3.593793870477057</v>
-      </c>
-      <c r="I15" t="n">
         <v>46.93431729914201</v>
       </c>
+      <c r="F15" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="H15" t="b">
+        <v>1</v>
+      </c>
+      <c r="I15" t="b">
+        <v>1</v>
+      </c>
       <c r="J15" t="n">
-        <v>2.000000000000002</v>
+        <v>100</v>
       </c>
       <c r="K15" t="n">
-        <v>2.000000000000002</v>
-      </c>
-      <c r="L15" t="b">
-        <v>1</v>
-      </c>
-      <c r="M15" t="b">
-        <v>1</v>
-      </c>
-      <c r="N15" t="n">
-        <v>100</v>
-      </c>
-      <c r="O15" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1101,41 +969,33 @@
         <v>2014</v>
       </c>
       <c r="B16" t="n">
-        <v>15.74490342470399</v>
+        <v>13.1228958335425</v>
       </c>
       <c r="C16" t="n">
-        <v>11.62549107212051</v>
+        <v>13.69</v>
       </c>
       <c r="D16" t="n">
-        <v>4.119412352583482</v>
+        <v>-0.5671041664575025</v>
       </c>
       <c r="E16" t="n">
-        <v>13.69</v>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="n">
-        <v>2.054903424703992</v>
-      </c>
-      <c r="I16" t="n">
         <v>49.07798020703141</v>
       </c>
+      <c r="F16" t="n">
+        <v>2.000000000000005</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2.000000000000005</v>
+      </c>
+      <c r="H16" t="b">
+        <v>1</v>
+      </c>
+      <c r="I16" t="b">
+        <v>1</v>
+      </c>
       <c r="J16" t="n">
-        <v>2.000000000000005</v>
+        <v>100</v>
       </c>
       <c r="K16" t="n">
-        <v>2.000000000000005</v>
-      </c>
-      <c r="L16" t="b">
-        <v>1</v>
-      </c>
-      <c r="M16" t="b">
-        <v>1</v>
-      </c>
-      <c r="N16" t="n">
-        <v>100</v>
-      </c>
-      <c r="O16" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1144,41 +1004,33 @@
         <v>2015</v>
       </c>
       <c r="B17" t="n">
-        <v>5.944329654724088</v>
+        <v>5.434349704276213</v>
       </c>
       <c r="C17" t="n">
-        <v>3.052323596362877</v>
+        <v>1.38</v>
       </c>
       <c r="D17" t="n">
-        <v>2.89200605836121</v>
+        <v>4.054349704276213</v>
       </c>
       <c r="E17" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="n">
-        <v>4.564329654724088</v>
-      </c>
-      <c r="I17" t="n">
         <v>50.13347864718618</v>
       </c>
+      <c r="F17" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="H17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" t="b">
+        <v>1</v>
+      </c>
       <c r="J17" t="n">
-        <v>2.000000000000002</v>
+        <v>100</v>
       </c>
       <c r="K17" t="n">
-        <v>2.000000000000002</v>
-      </c>
-      <c r="L17" t="b">
-        <v>1</v>
-      </c>
-      <c r="M17" t="b">
-        <v>1</v>
-      </c>
-      <c r="N17" t="n">
-        <v>100</v>
-      </c>
-      <c r="O17" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1187,41 +1039,33 @@
         <v>2016</v>
       </c>
       <c r="B18" t="n">
-        <v>12.91286635674778</v>
+        <v>10.82735287027742</v>
       </c>
       <c r="C18" t="n">
-        <v>9.921557709250674</v>
+        <v>11.96</v>
       </c>
       <c r="D18" t="n">
-        <v>2.991308647497103</v>
+        <v>-1.132647129722582</v>
       </c>
       <c r="E18" t="n">
-        <v>11.96</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="n">
-        <v>0.9528663567477746</v>
-      </c>
-      <c r="I18" t="n">
         <v>47.9578978407844</v>
       </c>
+      <c r="F18" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="H18" t="b">
+        <v>1</v>
+      </c>
+      <c r="I18" t="b">
+        <v>1</v>
+      </c>
       <c r="J18" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="K18" t="n">
-        <v>2.000000000000002</v>
-      </c>
-      <c r="L18" t="b">
-        <v>1</v>
-      </c>
-      <c r="M18" t="b">
-        <v>1</v>
-      </c>
-      <c r="N18" t="n">
-        <v>100</v>
-      </c>
-      <c r="O18" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1230,41 +1074,33 @@
         <v>2017</v>
       </c>
       <c r="B19" t="n">
-        <v>22.36374349342604</v>
+        <v>23.04668523976071</v>
       </c>
       <c r="C19" t="n">
-        <v>19.45016222066917</v>
+        <v>21.83</v>
       </c>
       <c r="D19" t="n">
-        <v>2.913581272756864</v>
+        <v>1.216685239760714</v>
       </c>
       <c r="E19" t="n">
-        <v>21.83</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="n">
-        <v>0.5337434934260408</v>
-      </c>
-      <c r="I19" t="n">
         <v>48.42161818409161</v>
       </c>
+      <c r="F19" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="H19" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" t="b">
+        <v>1</v>
+      </c>
       <c r="J19" t="n">
-        <v>2.000000000000004</v>
+        <v>100</v>
       </c>
       <c r="K19" t="n">
-        <v>2.000000000000002</v>
-      </c>
-      <c r="L19" t="b">
-        <v>1</v>
-      </c>
-      <c r="M19" t="b">
-        <v>1</v>
-      </c>
-      <c r="N19" t="n">
-        <v>100</v>
-      </c>
-      <c r="O19" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1273,41 +1109,33 @@
         <v>2018</v>
       </c>
       <c r="B20" t="n">
-        <v>-2.53417524006105</v>
+        <v>-2.53223033731219</v>
       </c>
       <c r="C20" t="n">
-        <v>-5.316577226565367</v>
+        <v>-4.38</v>
       </c>
       <c r="D20" t="n">
-        <v>2.782401986504317</v>
+        <v>1.84776966268781</v>
       </c>
       <c r="E20" t="n">
-        <v>-4.38</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="n">
-        <v>1.84582475993895</v>
-      </c>
-      <c r="I20" t="n">
         <v>47.43684633420839</v>
       </c>
+      <c r="F20" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.999999999999998</v>
+      </c>
+      <c r="H20" t="b">
+        <v>1</v>
+      </c>
+      <c r="I20" t="b">
+        <v>1</v>
+      </c>
       <c r="J20" t="n">
-        <v>2.000000000000004</v>
+        <v>100</v>
       </c>
       <c r="K20" t="n">
-        <v>1.999999999999998</v>
-      </c>
-      <c r="L20" t="b">
-        <v>1</v>
-      </c>
-      <c r="M20" t="b">
-        <v>1</v>
-      </c>
-      <c r="N20" t="n">
-        <v>100</v>
-      </c>
-      <c r="O20" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1316,41 +1144,33 @@
         <v>2019</v>
       </c>
       <c r="B21" t="n">
-        <v>32.74543223833429</v>
+        <v>32.55406884618817</v>
       </c>
       <c r="C21" t="n">
-        <v>29.61160825460702</v>
+        <v>31.49</v>
       </c>
       <c r="D21" t="n">
-        <v>3.133823983727269</v>
+        <v>1.064068846188167</v>
       </c>
       <c r="E21" t="n">
-        <v>31.49</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="n">
-        <v>1.25543223833429</v>
-      </c>
-      <c r="I21" t="n">
         <v>45.50548630255311</v>
       </c>
+      <c r="F21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" t="b">
+        <v>1</v>
+      </c>
       <c r="J21" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="K21" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" t="b">
-        <v>1</v>
-      </c>
-      <c r="M21" t="b">
-        <v>1</v>
-      </c>
-      <c r="N21" t="n">
-        <v>100</v>
-      </c>
-      <c r="O21" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1359,41 +1179,33 @@
         <v>2020</v>
       </c>
       <c r="B22" t="n">
-        <v>17.09049849505637</v>
+        <v>18.12353493137107</v>
       </c>
       <c r="C22" t="n">
-        <v>14.55480732304064</v>
+        <v>18.4</v>
       </c>
       <c r="D22" t="n">
-        <v>2.535691172015732</v>
+        <v>-0.2764650686289301</v>
       </c>
       <c r="E22" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="n">
-        <v>-1.309501504943629</v>
-      </c>
-      <c r="I22" t="n">
         <v>44.83786754564369</v>
       </c>
+      <c r="F22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2.000000000000005</v>
+      </c>
+      <c r="H22" t="b">
+        <v>1</v>
+      </c>
+      <c r="I22" t="b">
+        <v>1</v>
+      </c>
       <c r="J22" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="K22" t="n">
-        <v>2.000000000000005</v>
-      </c>
-      <c r="L22" t="b">
-        <v>1</v>
-      </c>
-      <c r="M22" t="b">
-        <v>1</v>
-      </c>
-      <c r="N22" t="n">
-        <v>100</v>
-      </c>
-      <c r="O22" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1402,41 +1214,33 @@
         <v>2021</v>
       </c>
       <c r="B23" t="n">
-        <v>29.17815654196793</v>
+        <v>27.09772981691429</v>
       </c>
       <c r="C23" t="n">
-        <v>26.89954276693625</v>
+        <v>28.71</v>
       </c>
       <c r="D23" t="n">
-        <v>2.278613775031675</v>
+        <v>-1.612270183085712</v>
       </c>
       <c r="E23" t="n">
-        <v>28.71</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="n">
-        <v>0.4681565419679252</v>
-      </c>
-      <c r="I23" t="n">
         <v>41.81514111784848</v>
       </c>
+      <c r="F23" t="n">
+        <v>2.000000000000005</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="H23" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" t="b">
+        <v>1</v>
+      </c>
       <c r="J23" t="n">
-        <v>2.000000000000005</v>
+        <v>100</v>
       </c>
       <c r="K23" t="n">
-        <v>2.000000000000004</v>
-      </c>
-      <c r="L23" t="b">
-        <v>1</v>
-      </c>
-      <c r="M23" t="b">
-        <v>1</v>
-      </c>
-      <c r="N23" t="n">
-        <v>100</v>
-      </c>
-      <c r="O23" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1445,41 +1249,33 @@
         <v>2022</v>
       </c>
       <c r="B24" t="n">
-        <v>-18.49776609950486</v>
+        <v>-18.38257793669661</v>
       </c>
       <c r="C24" t="n">
-        <v>-20.40946838321439</v>
+        <v>-18.11</v>
       </c>
       <c r="D24" t="n">
-        <v>1.911702283709529</v>
+        <v>-0.2725779366966066</v>
       </c>
       <c r="E24" t="n">
-        <v>-18.11</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="n">
-        <v>-0.3877660995048586</v>
-      </c>
-      <c r="I24" t="n">
         <v>41.60996806963041</v>
       </c>
+      <c r="F24" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" t="b">
+        <v>1</v>
+      </c>
+      <c r="I24" t="b">
+        <v>1</v>
+      </c>
       <c r="J24" t="n">
-        <v>2.000000000000002</v>
+        <v>100</v>
       </c>
       <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="b">
-        <v>1</v>
-      </c>
-      <c r="M24" t="b">
-        <v>1</v>
-      </c>
-      <c r="N24" t="n">
-        <v>100</v>
-      </c>
-      <c r="O24" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1488,41 +1284,33 @@
         <v>2023</v>
       </c>
       <c r="B25" t="n">
-        <v>30.8031440137597</v>
+        <v>28.99656497720724</v>
       </c>
       <c r="C25" t="n">
-        <v>28.34633877042602</v>
+        <v>26.29</v>
       </c>
       <c r="D25" t="n">
-        <v>2.456805243333683</v>
+        <v>2.70656497720724</v>
       </c>
       <c r="E25" t="n">
-        <v>26.29</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="n">
-        <v>4.513144013759703</v>
-      </c>
-      <c r="I25" t="n">
         <v>44.69222628835399</v>
       </c>
+      <c r="F25" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="H25" t="b">
+        <v>1</v>
+      </c>
+      <c r="I25" t="b">
+        <v>1</v>
+      </c>
       <c r="J25" t="n">
-        <v>2.000000000000004</v>
+        <v>100</v>
       </c>
       <c r="K25" t="n">
-        <v>2.000000000000004</v>
-      </c>
-      <c r="L25" t="b">
-        <v>1</v>
-      </c>
-      <c r="M25" t="b">
-        <v>1</v>
-      </c>
-      <c r="N25" t="n">
-        <v>100</v>
-      </c>
-      <c r="O25" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1531,41 +1319,33 @@
         <v>2024</v>
       </c>
       <c r="B26" t="n">
-        <v>27.67781993623965</v>
+        <v>26.72484234836757</v>
       </c>
       <c r="C26" t="n">
-        <v>25.89874324736693</v>
+        <v>25.02</v>
       </c>
       <c r="D26" t="n">
-        <v>1.779076688872725</v>
+        <v>1.704842348367571</v>
       </c>
       <c r="E26" t="n">
-        <v>25.02</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="n">
-        <v>2.657819936239655</v>
-      </c>
-      <c r="I26" t="n">
         <v>40.36115447201875</v>
       </c>
+      <c r="F26" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2.000000000000007</v>
+      </c>
+      <c r="H26" t="b">
+        <v>1</v>
+      </c>
+      <c r="I26" t="b">
+        <v>1</v>
+      </c>
       <c r="J26" t="n">
-        <v>2.000000000000004</v>
+        <v>100</v>
       </c>
       <c r="K26" t="n">
-        <v>2.000000000000007</v>
-      </c>
-      <c r="L26" t="b">
-        <v>1</v>
-      </c>
-      <c r="M26" t="b">
-        <v>1</v>
-      </c>
-      <c r="N26" t="n">
-        <v>100</v>
-      </c>
-      <c r="O26" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1574,41 +1354,33 @@
         <v>2025</v>
       </c>
       <c r="B27" t="n">
-        <v>19.6539137648381</v>
+        <v>19.50285254213123</v>
       </c>
       <c r="C27" t="n">
-        <v>18.3977558263514</v>
+        <v>17.88</v>
       </c>
       <c r="D27" t="n">
-        <v>1.256157938486705</v>
+        <v>1.622852542131231</v>
       </c>
       <c r="E27" t="n">
-        <v>17.88</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="n">
-        <v>1.773913764838099</v>
-      </c>
-      <c r="I27" t="n">
         <v>36.49727522889643</v>
       </c>
+      <c r="F27" t="n">
+        <v>2.000000000000002</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2.000000000000004</v>
+      </c>
+      <c r="H27" t="b">
+        <v>1</v>
+      </c>
+      <c r="I27" t="b">
+        <v>1</v>
+      </c>
       <c r="J27" t="n">
-        <v>2.000000000000002</v>
+        <v>100</v>
       </c>
       <c r="K27" t="n">
-        <v>2.000000000000004</v>
-      </c>
-      <c r="L27" t="b">
-        <v>1</v>
-      </c>
-      <c r="M27" t="b">
-        <v>1</v>
-      </c>
-      <c r="N27" t="n">
-        <v>100</v>
-      </c>
-      <c r="O27" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1680,13 +1452,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>677.4865391660518</v>
+        <v>602.1489317039319</v>
       </c>
       <c r="B2" t="n">
-        <v>8.207513726779991</v>
+        <v>7.784167267876363</v>
       </c>
       <c r="C2" t="n">
-        <v>24.64046501126234</v>
+        <v>-50.69714245085759</v>
       </c>
       <c r="D2" t="n">
         <v>652.8460741547894</v>

</xml_diff>